<commit_message>
Update wa-groove planning: upbeat lyrics sheet, pun titles, thumbnail prompts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S9ZzjqDoB7HA6WESKfKq7k
</commit_message>
<xml_diff>
--- a/wa_groove企画/wa_groove_characters.xlsx
+++ b/wa_groove企画/wa_groove_characters.xlsx
@@ -10,11 +10,13 @@
     <sheet name="キャラ一覧" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="共通スタイル" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="動画企画案" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="歌詞" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'キャラ一覧'!$A$1:$Q$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'共通スタイル'!$A$1:$C$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'動画企画案'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'共通スタイル'!$A$1:$C$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'動画企画案'!$A$1:$J$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'歌詞'!$A$1:$I$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2873,10 +2875,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="100" customWidth="1" min="3" max="3"/>
   </cols>
@@ -3153,8 +3155,59 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Suno共通タグ（歌入り版）</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>推奨タグ（歌詞シート用）</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 95–105 BPM, punchy boom bap drums, funky bassline, energetic, bright, head nod, Japanese lyrics（祭り系は taiko drums を追加）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Suno共通タグ（歌入り版）</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>声の指定</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>energetic male vocal または bright female vocal</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Suno共通タグ（歌入り版）</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>歌入り版で外すタグ</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>laid back, mellow, night, calm（※上の「避けるタグ（歌入り誘発）」はインスト版用）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C16"/>
+  <autoFilter ref="A1:C19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3165,17 +3218,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="90" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3216,7 +3271,17 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>元ネタ・洒落のポイント</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>サムネ案</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>サムネ用プロンプト（英語）</t>
         </is>
       </c>
     </row>
@@ -3251,12 +3316,22 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Rooftop Ninjas – Late Night Japanese Lo-fi to Study</t>
+          <t>忍ぶれど、ビートに出にけり屋根の上｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
+          <t>百人一首・平兼盛「忍ぶれど色に出でにけりわが恋は」のもじり。忍者なのにノリが隠せない</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
           <t>師弟の後ろ姿／満月／「深夜」</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi ninjas on a moonlit tiled rooftop: the rooftop ninja in indigo with a vermilion scarf wearing big headphones, the small apprentice ninja in matcha green holding a scroll, one ninja playing a shakuhachi, one tapping a small taiko drum, one spinning a vinyl record, one jumping high over a hemp plant. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -3291,12 +3366,22 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Samurai Crew – Japanese Boom Bap for Deep Focus</t>
+          <t>武士は食わねど、高ビート｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
+          <t>ことわざ「武士は食わねど高楊枝」の楊枝をビートに</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
           <t>隊長と若侍／夕焼けの城／「集中」</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi samurai jumping on stone steps of a castle town at sunset: the captain in an indigo haori with big headphones, the young samurai hugging a vinyl record, one holding a big rice ball, one beating a small taiko drum, one playing a shakuhachi, one waving a folding fan. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -3331,12 +3416,22 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Samurai Summer Break – Chill Japanese Beats</t>
+          <t>河童の川流れ、本日は侍も流されて｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
+          <t>ことわざ「河童の川流れ」×休日に流されるままの侍</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
           <t>縁側とスイカ／河童／「夏休み」</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: five chibi characters splashing at a summer riverside: the off-duty samurai in an indigo yukata waving an uchiwa fan, the kappa plucking an upright bass, one holding a slice of watermelon, one ringing a wind chime, one jumping with a cucumber, plus a friend with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -3371,12 +3466,22 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Midnight Yatai Session – Rainy Japanese Jazzhop</t>
+          <t>雨降って、ビート固まる深夜屋台｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
+          <t>ことわざ「雨降って地固まる」のもじり。雨上がりの屋台でセッションがまとまる</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
           <t>赤提灯／湯気／浪人の編笠</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters around a ramen stall at night after rain: the stall master tossing noodles with a strainer, the ronin DJ in a straw hat scratching a turntable, one slurping noodles, one playing a shamisen, one dancing with a paper umbrella, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -3411,12 +3516,22 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Temple Lo-fi – Mokugyo Beats to Relax &amp; Nap</t>
+          <t>門前の小僧、習わぬビートを刻む｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
+          <t>ことわざ「門前の小僧習わぬ経を読む」の経をビートに</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
           <t>木魚／眠る小僧と猫／桜</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: five chibi characters bouncing in a spring temple hall with cherry blossoms: the cheerful monk tapping a mokugyo, the novice monk boy hopping with a broom, a cat jumping, one monk ringing a small bell, one wearing big headphones and dancing. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -3451,12 +3566,22 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Matsuri Groove – Festival Japanese Beats</t>
+          <t>来年の話をしたら、鬼が踊りだした｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
+          <t>ことわざ「来年のことを言えば鬼が笑う」の「笑う」を「踊る」に</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
           <t>踊る連／太鼓の鬼／提灯</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi festival dancers on a lantern-lit street: the friendly oni beating a big taiko drum, Awa-odori dancers in indigo happi coats raising their hands, one waving an uchiwa fan, one ringing a kane bell, one playing a shinobue flute, one jumping with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -3491,12 +3616,22 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Kitsune Shrine – Sun Shower Japanese Jazzhop</t>
+          <t>狐の嫁入り、晴れときどき参列｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
+          <t>天気予報の「晴れときどき雨」×狐の嫁入りの参列</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
           <t>狐の行列／鳥居／和傘</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters in a shrine courtyard during a sun shower: the shrine maiden in vermilion hakama shaking kagura bells, a fox bride in white holding a vermilion umbrella, fox friends hopping with paper lanterns, one fox playing a shinobue flute, one twirling an umbrella, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -3531,12 +3666,22 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Heian Garden – Elegant Japanese Beats from Day to Night</t>
+          <t>春はあけぼの、夜は陰陽師｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
+          <t>枕草子「春はあけぼの」のもじり。昼は蹴鞠、夜は星読み</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
           <t>蹴鞠／藤棚／星空</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi Heian characters in a spring garden under wisteria: a noble in an indigo robe kicking a kemari ball high, the onmyoji with a small floating light, the festival child shaking a bell, one playing a koto, one dancing with a folding fan, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -3571,12 +3716,22 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>New Year Groove – Lucky Japanese Funk Beats</t>
+          <t>笑う門には、獅子きたる｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
+          <t>ことわざ「笑う門には福来る」の福を獅子舞に</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
           <t>獅子舞／若殿／「福」</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters at a New Year gate with pine decorations: the shishimai lion dancer snapping its jaws, the young lord in a vermilion kamishimo jumping, the maneki-neko cat beckoning, one retainer beating a small taiko drum, one playing a shinobue flute, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -3611,17 +3766,722 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Edo Night Theater – Shamisen &amp; Biwa Jazzhop</t>
+          <t>祇園精舎の鐘の声、本日はビートの声｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
+          <t>平家物語の冒頭「祇園精舎の鐘の声」を琵琶法師がビートで語る</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
           <t>三味線／隈取／提灯</t>
         </is>
       </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi performers on a wooden theater stage lined with lanterns: the kabuki actor with kumadori makeup striking a pose, an elegant musician lady in modest fully covered kimono playing a shamisen, the biwa player strumming, one clapping hyoshigi wooden clappers, one beating a small taiko drum, one jumping with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H11"/>
+  <autoFilter ref="A1:J11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>企画No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>曲タイトル</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>元ネタ・洒落のポイント</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>登場キャラ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>題材の伝承・物語</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>BPM</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Suno スタイル（英語）</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>歌詞（Suno Lyrics欄に貼る）</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>lyricsファイル名</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>麻とびこえて、きょうもワンステップ</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>忍者の「麻跳び」修行×ステップアップの掛け言葉</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>屋根の上の忍者（ヘッドホン）、見習い忍者</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>忍者は麻を植え、毎日伸びる麻を跳び越えて跳躍力を鍛えたという言い伝え</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 100 BPM, punchy boom bap drums, funky bassline, Japanese shakuhachi, Japanese shamisen, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>[Verse]
+やねのうえ　つきが　まるい
+ヘッドホンから　かぜの　おと
+ししょうは　だまって　ゆびさした
+きょうも　あさを　とびこえろ
+[Chorus]
+とんで（はっ）　はねて（それ）　あさを　こえろ
+きのうより　すこし　たかく　なれ
+まわって　すべって　かわらの　うえ
+しのびあしで　ビートに　のれ
+[Verse]
+たねを　まいた　あの　ひから
+あさは　まいにち　のびていく
+おいらの　あしも　まけないで
+まいにち　ひとつ　ステップアップ
+[Chorus]
+とんで（はっ）　はねて（それ）　あさを　こえろ
+きのうより　すこし　たかく　なれ
+まわって　すべって　かわらの　うえ
+しのびあしで　ビートに　のれ
+[Outro]
+しのぶれど（はっ）　でちゃうんだ（それ）</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>01_麻とびこえて、きょうもワンステップ.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>腹が減っては、ビートはできぬ</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ことわざ「腹が減っては戦ができぬ」のもじり</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>侍集団の隊長、若侍（レコードを抱える）</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>戦の前に握り飯で腹ごしらえをした武士たち。腹ごしらえは何よりの備え</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>96</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 96 BPM, punchy boom bap drums, funky bassline, Japanese shamisen, Japanese shakuhachi, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>[Verse]
+いしだんに　ならんで　すわる
+ゆうやけ　しろの　かげが　のびる
+たいちょうが　つつみを　ひらいたら
+おおきな　おむすび　ふたつ
+[Chorus]
+ほおばれ（よいしょ）　たちあがれ（それ）
+はらが　へっては　ビートは　できぬ
+ふんで　ならして　いしだんを
+いっぽ　いっぽ　かけあがれ
+[Verse]
+わかざむらいは　レコードを
+かたなの　かわりに　だいじに　かかえ
+はりを　おとせば　まちが　おどる
+たいちょうの　くびも　ゆれだした
+[Chorus]
+ほおばれ（よいしょ）　たちあがれ（それ）
+はらが　へっては　ビートは　できぬ
+ふんで　ならして　いしだんを
+いっぽ　いっぽ　かけあがれ</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>02_腹が減っては、ビートはできぬ.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>鬼に金棒、河童にベース</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ことわざ「鬼に金棒」のもじり。河童にはウッドベースが最強の相棒</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>侍の休日（浴衣で縁側）、河童（追加）</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>河童は頭の皿の水が乾くと力が抜け、きゅうりが大好物という伝承</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 98 BPM, punchy boom bap drums, funky bassline, Japanese koto, Japanese shamisen, bright female vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>[Verse]
+えんがわで　うちわを　ぱたぱた
+すいかの　たねを　とばしたら
+かわの　ほうから　ぼん　ぼん　ぼん
+かっぱが　ベースを　はじいてる
+[Chorus]
+はじけ（はっ）　はねろ（それ）　みずしぶき
+おにに　かなぼう　かっぱに　ベース
+まわれ　まわれ　かざぐるま
+なつやすみは　まだ　おわらない
+[Verse]
+おさらの　みずが　ひからぬように
+ときどき　かわへ　とびこんで
+きゅうりを　かじって　ひとやすみ
+さむらいも　はだしで　かけだした
+[Chorus]
+はじけ（はっ）　はねろ（それ）　みずしぶき
+おにに　かなぼう　かっぱに　ベース
+まわれ　まわれ　かざぐるま
+なつやすみは　まだ　おわらない</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>03_鬼に金棒、河童にベース.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>二八そばより、十六ビート</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>江戸の「二八そば」は2×8＝16。そばの値段と16ビートの掛け算洒落</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>屋台の大将、浪人DJ</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>江戸の夜鳴きそば。二八そばは「十六文」の値段から来たという説がある</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 100 BPM, punchy boom bap drums, funky bassline, Japanese shamisen, Japanese shakuhachi, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>[Verse]
+あめあがり　あかちょうちん
+ゆげの　むこうに　あみがさ　ひとつ
+たいしょうが　めんを　ちゃっ　ちゃっ　ちゃっ
+ろうにんは　さらを　くる　くる　くる
+[Chorus]
+きざめ（はっ）　ゆらせ（それ）　よるの　まち
+にはちそばより　じゅうろくビート
+まわせ　まわせ　にまいの　さら
+どんぶりも　レコードも　あつあつだ
+[Verse]
+にはちで　じゅうろく　かけざんで
+えどの　よなきそば　うたいだす
+みずたまり　はねて　げたが　なる
+あさまで　のれんは　おろさない
+[Chorus]
+きざめ（はっ）　ゆらせ（それ）　よるの　まち
+にはちそばより　じゅうろくビート
+まわせ　まわせ　にまいの　さら
+どんぶりも　レコードも　あつあつだ</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>04_二八そばより、十六ビート.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>魚は眠らず、小僧は眠る</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>木魚の由来（魚は眠らない）と昼寝する小僧の対比</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>木魚ビート僧、昼寝する小僧さん</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>魚は昼も夜も目を閉じないことから、眠らず修行に励めという戒めで木魚が魚の形になったという説</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>96</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 96 BPM, punchy boom bap drums, funky bassline, Japanese shakuhachi, Japanese koto, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>[Verse]
+ぽく　ぽく　ぽく　と　ほんどうに
+もくぎょの　ビートが　ひびいてる
+さかなは　ねむらず　めを　あけて
+なまけちゃ　だめだと　いうけれど
+[Chorus]
+たたけ（はっ）　うなずけ（それ）　ぽく　ぽく　ぽん
+さかなは　ねむらず　こぞうは　ねむる
+さくら　ひらひら　まいおりて
+ゆめの　なかでも　ステップ　ふむ
+[Verse]
+えんがわで　ねこと　まるくなり
+ほうきを　まくらに　すう　すう　すう
+もんぜんの　こぞうは　ならわずに
+ねごとで　ビートを　きざんでる
+[Chorus]
+たたけ（はっ）　うなずけ（それ）　ぽく　ぽく　ぽん
+さかなは　ねむらず　こぞうは　ねむる
+さくら　ひらひら　まいおりて
+ゆめの　なかでも　ステップ　ふむ</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>05_魚は眠らず、小僧は眠る.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>踊る阿呆に、太鼓たたく鬼</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>阿波踊りの「踊る阿呆に見る阿呆」の「見る阿呆」を太鼓の鬼に</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>阿波踊り連、太鼓の鬼</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>阿波踊りのよしこの節と、鬼の面で太鼓を打つ佐渡の「鬼太鼓」</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>104</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 104 BPM, punchy boom bap drums, funky bassline, Japanese shinobue, Japanese shamisen, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>[Verse]
+ちょうちんの　あかりが　つづく　みち
+てを　あげて　あしを　ふみだせば
+やまの　やぐらで　どーん　どーん
+おにが　たいこを　たたいてる
+[Chorus]
+えらいやっちゃ（はっ）　よいよいよい（それ）
+おどる　あほうに　たいこ　たたく　おに
+まわれ　はねろ　てを　ふれ
+おなじ　あほなら　おどらにゃ　そんそん
+[Verse]
+こわい　かおして　めは　にこにこ
+つのも　ゆれてる　リズムに　のって
+こどもも　ねこも　おばあちゃんも
+ひとつの　わに　なって　まわる
+[Chorus]
+えらいやっちゃ（はっ）　よいよいよい（それ）
+おどる　あほうに　たいこ　たたく　おに
+まわれ　はねろ　てを　ふれ
+おなじ　あほなら　おどらにゃ　そんそん</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>06_踊る阿呆に、太鼓たたく鬼.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>お天気雨は、狐の招待状</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>天気雨＝狐の嫁入りの伝承を「招待状」に見立てた</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>巫女、狐の嫁入り</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>晴れているのに雨が降るのは、狐が嫁入り行列を人に見られないようにするためという伝承</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>96</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 96 BPM, punchy boom bap drums, funky bassline, Japanese koto, Japanese shinobue, bright female vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>[Verse]
+はれているのに　ぽつ　ぽつ　ぽつ
+とりいの　むこうが　きらきら　ひかる
+みこさん　ほうきを　とめて　みた
+ちょうちん　ゆらゆら　ぎょうれつだ
+[Chorus]
+しゃらん（はっ）　しゃらん（それ）　すずが　なる
+おてんきあめは　きつねの　しょうたいじょう
+くるり　まわして　あかい　かさ
+はねて　わらって　はれのち　あめ
+[Verse]
+しろい　きものの　はなよめさん
+しっぽを　そっと　かくしてる
+みつけても　ないしょに　しておこう
+にじが　かかれば　おひらきだ
+[Chorus]
+しゃらん（はっ）　しゃらん（それ）　すずが　なる
+おてんきあめは　きつねの　しょうたいじょう
+くるり　まわして　あかい　かさ
+はねて　わらって　はれのち　あめ</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>07_お天気雨は、狐の招待状.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>いとをかし、いとグルーヴィ</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>枕草子の「いとをかし」に今っぽい「グルーヴィ」を重ねた</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>平安貴族（蹴鞠）、陰陽師、稚児</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>蹴鞠では「アリ」「ヤア」「オウ」と声をかけ合う。鞠の精の名に由来するという言い伝え</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 98 BPM, punchy boom bap drums, funky bassline, Japanese koto, Japanese ryuteki flute, bright female vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>[Verse]
+ふじの　はなが　ゆれる　にわ
+きぬの　そでを　ひるがえし
+まりを　ぽーんと　けりあげて
+おちないように　そらへ　かえす
+[Chorus]
+ありー（はっ）　やあ（それ）　おう（よいしょ）
+いとをかし　いとグルーヴィ
+けって　はねて　くるりと　まわれ
+まりは　ひるまの　おつきさま
+[Verse]
+よるが　くれば　おんみょうじ
+ほしを　かぞえて　うらなえば
+あしたも　はれて　まりびより
+ちごも　すずを　しゃんと　ふる
+[Chorus]
+ありー（はっ）　やあ（それ）　おう（よいしょ）
+いとをかし　いとグルーヴィ
+けって　はねて　くるりと　まわれ
+まりは　ひるまの　おつきさま</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>08_いとをかし、いとグルーヴィ.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>猫の手も、招きたいお正月</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>慣用句「猫の手も借りたい」×招き猫の手招き</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>獅子舞、若殿と家臣団、招き猫（追加）</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>獅子舞に頭を噛まれると邪気が払われ無病息災に。招き猫は右手でお金、左手で人を招くといわれる</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 102 BPM, punchy boom bap drums, funky bassline, Japanese shinobue, Japanese shamisen, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>[Verse]
+おしょうがつ　まつかざりの　もん
+わかとの　ねぼうで　おおさわぎ
+かしんが　ばたばた　はしる　なか
+ししまいが　ぱくぱく　やってきた
+[Chorus]
+かぷっと（はっ）　かまれて（それ）　ふくが　くる
+ねこの　ても　まねきたい　いそがしさ
+まわれ　おどれ　ししがしら
+ことしも　げんきに　いきましょう
+[Verse]
+しょうてんがいの　まねきねこ
+みぎてで　おかね　ひだりで　ひと
+わかとのも　まねして　てを　ふれば
+えがおが　ぞろぞろ　あつまった
+[Chorus]
+かぷっと（はっ）　かまれて（それ）　ふくが　くる
+ねこの　ても　まねきたい　いそがしさ
+まわれ　おどれ　ししがしら
+ことしも　げんきに　いきましょう</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>09_猫の手も、招きたいお正月.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>待ってました、と言わせたい</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>歌舞伎の大向う（客席からの掛け声）「待ってました！」</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>花魁（三味線持ち）、歌舞伎役者、琵琶法師（追加）</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>歌舞伎の客席から飛ぶ大向うの掛け声と、平家物語を語り継いだ琵琶法師</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 98 BPM, punchy boom bap drums, funky bassline, Japanese shamisen, Japanese biwa, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>[Verse]
+ひょうしぎ　かん　かん　まくが　あく
+ちょうちん　ならぶ　しばいごや
+しゃみせん　べんべん　たかなれば
+びわの　ねいろが　ものがたる
+[Chorus]
+よっ（はっ）　まってました（それ）
+みえを　きるまで　あと　すこし
+まわって　ふんで　とん　とん　とん
+まってましたと　いわせたい
+[Verse]
+ぎおんしょうじゃの　かねの　こえ
+むかしの　はなしを　いまふうに
+ちょんまげ　ゆらして　くびを　ふり
+おおむこう　こえが　かかったら
+[Chorus]
+よっ（はっ）　まってました（それ）
+みえを　きるまで　あと　すこし
+まわって　ふんで　とん　とん　とん
+まってましたと　いわせたい</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>10_待ってました、と言わせたい.txt</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add how-to and copy-paste sheets, color-code Suno/ChatGPT columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S9ZzjqDoB7HA6WESKfKq7k
</commit_message>
<xml_diff>
--- a/wa_groove企画/wa_groove_characters.xlsx
+++ b/wa_groove企画/wa_groove_characters.xlsx
@@ -7,16 +7,18 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="キャラ一覧" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="共通スタイル" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="動画企画案" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="歌詞" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="使い方" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="コピペ早見表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="キャラ一覧" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="共通スタイル" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="動画企画案" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="歌詞" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'キャラ一覧'!$A$1:$Q$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'共通スタイル'!$A$1:$C$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'動画企画案'!$A$1:$J$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'歌詞'!$A$1:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'キャラ一覧'!$A$1:$Q$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'共通スタイル'!$A$1:$C$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'動画企画案'!$A$1:$J$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'歌詞'!$A$1:$I$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +45,29 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002E4A62"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -54,6 +77,26 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E4A62"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C55A11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -92,6 +135,33 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -456,6 +526,817 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002E4A62"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>このファイルの使い方</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>このファイル1つで全部見られます。下のタブ（シート）を切り替えてください。CSVと lyrics フォルダは予備なので開かなくてOKです。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>シート一覧</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>コピペ早見表 … 企画ごとに、SunoとChatGPTに貼るものだけを横一列にまとめた表。普段はここだけ見ればOK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>キャラ一覧 … 27キャラの設定。キャラ単体の画像を作るときは緑の列をコピペ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>共通スタイル … 絵柄をそろえるコツ、Sunoのタグ集</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>動画企画案 … 10本の企画、動画タイトル、サムネ用プロンプト</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>歌詞 … 10曲の歌詞・元ネタ・伝承</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>色の見方</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>オレンジの列 ＝ Suno に貼る</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>緑の列 ＝ ChatGPT に貼る（画像生成）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Sunoで1曲作る手順（コピペ早見表を使用）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>1. Sunoで「Custom」モードにする（Instrumental はオフ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2. ① をコピー → Title 欄に貼る</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>3. ② をコピー → Style of Music 欄に貼る</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>4. ③ をコピー → Lyrics 欄に貼る</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>5. Create を押す（2曲できるので良いほうを残す）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>ChatGPTでサムネを作る手順</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>1. ChatGPTで新しいチャットを開く</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>2. ④ をコピーして貼り、送信する</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>3. 文字（タイトル）はCanvaなどで左上の空きスペースに後から入れる</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>★ コピペのコツ（重要）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>歌詞のように改行があるセルは、セルを選んでCtrl+Cすると前後に " が付くことがあります。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>→ セルをダブルクリック（またはF2）→ Ctrl+A で中身を全選択 → Ctrl+C でコピーすると、" が付きません。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>→ Googleスプレッドシートで見る場合は、このxlsxをGoogleドライブにアップして開くとシートの切り替えもそのまま使えます。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C55A11"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>企画No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>登場キャラ</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>① 【Suno】Title欄</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>② 【Suno】Style欄</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>③ 【Suno】Lyrics欄</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>④ 【ChatGPT】サムネ画像</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>⑤ 【YouTube】動画タイトル</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>屋根の上の忍者（ヘッドホン）、見習い忍者</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>麻とびこえて、きょうもワンステップ</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 100 BPM, punchy boom bap drums, funky bassline, Japanese shakuhachi, Japanese shamisen, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>[Verse]
+やねのうえ　つきが　まるい
+ヘッドホンから　かぜの　おと
+ししょうは　だまって　ゆびさした
+きょうも　あさを　とびこえろ
+[Chorus]
+とんで（はっ）　はねて（それ）　あさを　こえろ
+きのうより　すこし　たかく　なれ
+まわって　すべって　かわらの　うえ
+しのびあしで　ビートに　のれ
+[Verse]
+たねを　まいた　あの　ひから
+あさは　まいにち　のびていく
+おいらの　あしも　まけないで
+まいにち　ひとつ　ステップアップ
+[Chorus]
+とんで（はっ）　はねて（それ）　あさを　こえろ
+きのうより　すこし　たかく　なれ
+まわって　すべって　かわらの　うえ
+しのびあしで　ビートに　のれ
+[Outro]
+しのぶれど（はっ）　でちゃうんだ（それ）</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi ninjas on a moonlit tiled rooftop: the rooftop ninja in indigo with a vermilion scarf wearing big headphones, the small apprentice ninja in matcha green holding a scroll, one ninja playing a shakuhachi, one tapping a small taiko drum, one spinning a vinyl record, one jumping high over a hemp plant. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>忍ぶれど、ビートに出にけり屋根の上｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>侍集団の隊長、若侍（レコードを抱える）</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>腹が減っては、ビートはできぬ</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 96 BPM, punchy boom bap drums, funky bassline, Japanese shamisen, Japanese shakuhachi, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>[Verse]
+いしだんに　ならんで　すわる
+ゆうやけ　しろの　かげが　のびる
+たいちょうが　つつみを　ひらいたら
+おおきな　おむすび　ふたつ
+[Chorus]
+ほおばれ（よいしょ）　たちあがれ（それ）
+はらが　へっては　ビートは　できぬ
+ふんで　ならして　いしだんを
+いっぽ　いっぽ　かけあがれ
+[Verse]
+わかざむらいは　レコードを
+かたなの　かわりに　だいじに　かかえ
+はりを　おとせば　まちが　おどる
+たいちょうの　くびも　ゆれだした
+[Chorus]
+ほおばれ（よいしょ）　たちあがれ（それ）
+はらが　へっては　ビートは　できぬ
+ふんで　ならして　いしだんを
+いっぽ　いっぽ　かけあがれ</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi samurai jumping on stone steps of a castle town at sunset: the captain in an indigo haori with big headphones, the young samurai hugging a vinyl record, one holding a big rice ball, one beating a small taiko drum, one playing a shakuhachi, one waving a folding fan. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>武士は食わねど、高ビート｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>侍の休日（浴衣で縁側）、河童（追加）</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>鬼に金棒、河童にベース</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 98 BPM, punchy boom bap drums, funky bassline, Japanese koto, Japanese shamisen, bright female vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>[Verse]
+えんがわで　うちわを　ぱたぱた
+すいかの　たねを　とばしたら
+かわの　ほうから　ぼん　ぼん　ぼん
+かっぱが　ベースを　はじいてる
+[Chorus]
+はじけ（はっ）　はねろ（それ）　みずしぶき
+おにに　かなぼう　かっぱに　ベース
+まわれ　まわれ　かざぐるま
+なつやすみは　まだ　おわらない
+[Verse]
+おさらの　みずが　ひからぬように
+ときどき　かわへ　とびこんで
+きゅうりを　かじって　ひとやすみ
+さむらいも　はだしで　かけだした
+[Chorus]
+はじけ（はっ）　はねろ（それ）　みずしぶき
+おにに　かなぼう　かっぱに　ベース
+まわれ　まわれ　かざぐるま
+なつやすみは　まだ　おわらない</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: five chibi characters splashing at a summer riverside: the off-duty samurai in an indigo yukata waving an uchiwa fan, the kappa plucking an upright bass, one holding a slice of watermelon, one ringing a wind chime, one jumping with a cucumber, plus a friend with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>河童の川流れ、本日は侍も流されて｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>屋台の大将、浪人DJ</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>二八そばより、十六ビート</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 100 BPM, punchy boom bap drums, funky bassline, Japanese shamisen, Japanese shakuhachi, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>[Verse]
+あめあがり　あかちょうちん
+ゆげの　むこうに　あみがさ　ひとつ
+たいしょうが　めんを　ちゃっ　ちゃっ　ちゃっ
+ろうにんは　さらを　くる　くる　くる
+[Chorus]
+きざめ（はっ）　ゆらせ（それ）　よるの　まち
+にはちそばより　じゅうろくビート
+まわせ　まわせ　にまいの　さら
+どんぶりも　レコードも　あつあつだ
+[Verse]
+にはちで　じゅうろく　かけざんで
+えどの　よなきそば　うたいだす
+みずたまり　はねて　げたが　なる
+あさまで　のれんは　おろさない
+[Chorus]
+きざめ（はっ）　ゆらせ（それ）　よるの　まち
+にはちそばより　じゅうろくビート
+まわせ　まわせ　にまいの　さら
+どんぶりも　レコードも　あつあつだ</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters around a ramen stall at night after rain: the stall master tossing noodles with a strainer, the ronin DJ in a straw hat scratching a turntable, one slurping noodles, one playing a shamisen, one dancing with a paper umbrella, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>雨降って、ビート固まる深夜屋台｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>木魚ビート僧、昼寝する小僧さん</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>魚は眠らず、小僧は眠る</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 96 BPM, punchy boom bap drums, funky bassline, Japanese shakuhachi, Japanese koto, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>[Verse]
+ぽく　ぽく　ぽく　と　ほんどうに
+もくぎょの　ビートが　ひびいてる
+さかなは　ねむらず　めを　あけて
+なまけちゃ　だめだと　いうけれど
+[Chorus]
+たたけ（はっ）　うなずけ（それ）　ぽく　ぽく　ぽん
+さかなは　ねむらず　こぞうは　ねむる
+さくら　ひらひら　まいおりて
+ゆめの　なかでも　ステップ　ふむ
+[Verse]
+えんがわで　ねこと　まるくなり
+ほうきを　まくらに　すう　すう　すう
+もんぜんの　こぞうは　ならわずに
+ねごとで　ビートを　きざんでる
+[Chorus]
+たたけ（はっ）　うなずけ（それ）　ぽく　ぽく　ぽん
+さかなは　ねむらず　こぞうは　ねむる
+さくら　ひらひら　まいおりて
+ゆめの　なかでも　ステップ　ふむ</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: five chibi characters bouncing in a spring temple hall with cherry blossoms: the cheerful monk tapping a mokugyo, the novice monk boy hopping with a broom, a cat jumping, one monk ringing a small bell, one wearing big headphones and dancing. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>門前の小僧、習わぬビートを刻む｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>阿波踊り連、太鼓の鬼</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>踊る阿呆に、太鼓たたく鬼</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 104 BPM, punchy boom bap drums, funky bassline, Japanese shinobue, Japanese shamisen, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>[Verse]
+ちょうちんの　あかりが　つづく　みち
+てを　あげて　あしを　ふみだせば
+やまの　やぐらで　どーん　どーん
+おにが　たいこを　たたいてる
+[Chorus]
+えらいやっちゃ（はっ）　よいよいよい（それ）
+おどる　あほうに　たいこ　たたく　おに
+まわれ　はねろ　てを　ふれ
+おなじ　あほなら　おどらにゃ　そんそん
+[Verse]
+こわい　かおして　めは　にこにこ
+つのも　ゆれてる　リズムに　のって
+こどもも　ねこも　おばあちゃんも
+ひとつの　わに　なって　まわる
+[Chorus]
+えらいやっちゃ（はっ）　よいよいよい（それ）
+おどる　あほうに　たいこ　たたく　おに
+まわれ　はねろ　てを　ふれ
+おなじ　あほなら　おどらにゃ　そんそん</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi festival dancers on a lantern-lit street: the friendly oni beating a big taiko drum, Awa-odori dancers in indigo happi coats raising their hands, one waving an uchiwa fan, one ringing a kane bell, one playing a shinobue flute, one jumping with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>来年の話をしたら、鬼が踊りだした｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>巫女、狐の嫁入り</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>お天気雨は、狐の招待状</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 96 BPM, punchy boom bap drums, funky bassline, Japanese koto, Japanese shinobue, bright female vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>[Verse]
+はれているのに　ぽつ　ぽつ　ぽつ
+とりいの　むこうが　きらきら　ひかる
+みこさん　ほうきを　とめて　みた
+ちょうちん　ゆらゆら　ぎょうれつだ
+[Chorus]
+しゃらん（はっ）　しゃらん（それ）　すずが　なる
+おてんきあめは　きつねの　しょうたいじょう
+くるり　まわして　あかい　かさ
+はねて　わらって　はれのち　あめ
+[Verse]
+しろい　きものの　はなよめさん
+しっぽを　そっと　かくしてる
+みつけても　ないしょに　しておこう
+にじが　かかれば　おひらきだ
+[Chorus]
+しゃらん（はっ）　しゃらん（それ）　すずが　なる
+おてんきあめは　きつねの　しょうたいじょう
+くるり　まわして　あかい　かさ
+はねて　わらって　はれのち　あめ</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters in a shrine courtyard during a sun shower: the shrine maiden in vermilion hakama shaking kagura bells, a fox bride in white holding a vermilion umbrella, fox friends hopping with paper lanterns, one fox playing a shinobue flute, one twirling an umbrella, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>狐の嫁入り、晴れときどき参列｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>平安貴族（蹴鞠）、陰陽師、稚児</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>いとをかし、いとグルーヴィ</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 98 BPM, punchy boom bap drums, funky bassline, Japanese koto, Japanese ryuteki flute, bright female vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>[Verse]
+ふじの　はなが　ゆれる　にわ
+きぬの　そでを　ひるがえし
+まりを　ぽーんと　けりあげて
+おちないように　そらへ　かえす
+[Chorus]
+ありー（はっ）　やあ（それ）　おう（よいしょ）
+いとをかし　いとグルーヴィ
+けって　はねて　くるりと　まわれ
+まりは　ひるまの　おつきさま
+[Verse]
+よるが　くれば　おんみょうじ
+ほしを　かぞえて　うらなえば
+あしたも　はれて　まりびより
+ちごも　すずを　しゃんと　ふる
+[Chorus]
+ありー（はっ）　やあ（それ）　おう（よいしょ）
+いとをかし　いとグルーヴィ
+けって　はねて　くるりと　まわれ
+まりは　ひるまの　おつきさま</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi Heian characters in a spring garden under wisteria: a noble in an indigo robe kicking a kemari ball high, the onmyoji with a small floating light, the festival child shaking a bell, one playing a koto, one dancing with a folding fan, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>春はあけぼの、夜は陰陽師｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>獅子舞、若殿と家臣団、招き猫（追加）</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>猫の手も、招きたいお正月</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 102 BPM, punchy boom bap drums, funky bassline, Japanese shinobue, Japanese shamisen, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>[Verse]
+おしょうがつ　まつかざりの　もん
+わかとの　ねぼうで　おおさわぎ
+かしんが　ばたばた　はしる　なか
+ししまいが　ぱくぱく　やってきた
+[Chorus]
+かぷっと（はっ）　かまれて（それ）　ふくが　くる
+ねこの　ても　まねきたい　いそがしさ
+まわれ　おどれ　ししがしら
+ことしも　げんきに　いきましょう
+[Verse]
+しょうてんがいの　まねきねこ
+みぎてで　おかね　ひだりで　ひと
+わかとのも　まねして　てを　ふれば
+えがおが　ぞろぞろ　あつまった
+[Chorus]
+かぷっと（はっ）　かまれて（それ）　ふくが　くる
+ねこの　ても　まねきたい　いそがしさ
+まわれ　おどれ　ししがしら
+ことしも　げんきに　いきましょう</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters at a New Year gate with pine decorations: the shishimai lion dancer snapping its jaws, the young lord in a vermilion kamishimo jumping, the maneki-neko cat beckoning, one retainer beating a small taiko drum, one playing a shinobue flute, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>笑う門には、獅子きたる｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>花魁（三味線持ち）、歌舞伎役者、琵琶法師（追加）</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>待ってました、と言わせたい</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Japanese jazzy hip hop, upbeat groove, 98 BPM, punchy boom bap drums, funky bassline, Japanese shamisen, Japanese biwa, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>[Verse]
+ひょうしぎ　かん　かん　まくが　あく
+ちょうちん　ならぶ　しばいごや
+しゃみせん　べんべん　たかなれば
+びわの　ねいろが　ものがたる
+[Chorus]
+よっ（はっ）　まってました（それ）
+みえを　きるまで　あと　すこし
+まわって　ふんで　とん　とん　とん
+まってましたと　いわせたい
+[Verse]
+ぎおんしょうじゃの　かねの　こえ
+むかしの　はなしを　いまふうに
+ちょんまげ　ゆらして　くびを　ふり
+おおむこう　こえが　かかったら
+[Chorus]
+よっ（はっ）　まってました（それ）
+みえを　きるまで　あと　すこし
+まわって　ふんで　とん　とん　とん
+まってましたと　いわせたい</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi performers on a wooden theater stage lined with lanterns: the kabuki actor with kumadori makeup striking a pose, an elegant musician lady in modest fully covered kimono playing a shamisen, the biwa player strumming, one clapping hyoshigi wooden clappers, one beating a small taiko drum, one jumping with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>祇園精舎の鐘の声、本日はビートの声｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -542,14 +1423,14 @@
           <t>雰囲気・聴く場面</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Suno用プロンプト</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>画像生成プロンプト</t>
+      <c r="M1" s="9" t="inlineStr">
+        <is>
+          <t>【Suno】Style欄にコピペ（インスト版）</t>
+        </is>
+      </c>
+      <c r="N1" s="10" t="inlineStr">
+        <is>
+          <t>【ChatGPT】キャラ画像プロンプト（コピペ）</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
@@ -627,12 +1508,12 @@
           <t>集中作業・勉強</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="11" t="inlineStr">
         <is>
           <t>Japanese boom bap, dusty drums, shakuhachi melody, shamisen plucks, taiko accents, warm vinyl crackle, steady head-nod groove, 88 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A calm samurai captain in an indigo haori with vermilion cords and mustard hakama, arms crossed, sitting on stone steps of a castle town at dusk with his crew behind him, headphones around his neck.</t>
         </is>
@@ -712,12 +1593,12 @@
           <t>朝・作業・読書</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M3" s="11" t="inlineStr">
         <is>
           <t>Japanese jazzhop, mellow rhodes chords, koto riffs, upright bass, soft swung drums, vinyl crackle, cozy morning feel, 82 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="N3" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A young samurai boy in a matcha green kimono and indigo hakama hugging a vinyl record with a happy face, standing in front of an old antique shop with crates of records.</t>
         </is>
@@ -797,12 +1678,12 @@
           <t>夜・ドライブ</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" s="11" t="inlineStr">
         <is>
           <t>gritty Japanese boom bap, chopped shamisen samples, record scratches, deep kick, shakuhachi breath, moonlit night vibe, 92 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="N4" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A cool wandering ronin DJ wearing a faded indigo kimono and woven straw hat, scratching a wooden turntable on a riverbank under a full moon.</t>
         </is>
@@ -882,12 +1763,12 @@
           <t>夏の昼・リラックス</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M5" s="11" t="inlineStr">
         <is>
           <t>chill Japanese jazzhop, lazy summer afternoon, koto and nylon guitar, soft rhodes, wind chime ambience, gentle brushed drums, 75 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="N5" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. An off-duty samurai relaxing on a wooden engawa porch in an indigo yukata with flowing-water pattern, fanning himself with an uchiwa, slice of watermelon and wind chime nearby, morning glories in the garden.</t>
         </is>
@@ -967,12 +1848,12 @@
           <t>朝の家事・気分上げ</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M6" s="11" t="inlineStr">
         <is>
           <t>upbeat Japanese funk-hop groove, slap bass, clavinet, tsuzumi hand drums, shinobue flute riffs, playful bouncy rhythm, 98 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="N6" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A cheeky young lord in a vermilion kamishimo tapping a folding fan, surrounded by nodding retainers in indigo and mustard kamishimo, inside a castle hall with shoji light.</t>
         </is>
@@ -1052,12 +1933,12 @@
           <t>気分を上げたい時・掃除</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M7" s="11" t="inlineStr">
         <is>
           <t>festive Japanese breakbeat groove, kane bell, shime-daiko, shinobue melody, shamisen strums, funky bass, joyful dance energy, 104 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="N7" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. An Awa-odori dance troupe of chibi dancers in indigo happi coats and straw hats, raising hands in rhythm on a festival street lined with glowing paper lanterns.</t>
         </is>
@@ -1137,12 +2018,12 @@
           <t>夜・読書</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M8" s="11" t="inlineStr">
         <is>
           <t>elegant Japanese jazzhop, refined shamisen phrases, koto, upright bass, rhodes piano, soft lantern-lit night mood, 78 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="N8" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. An elegant musician lady in modest layered kimono of indigo and vermilion, fully covered, calm dignified smile, playing shamisen in a tatami room lit by an andon lantern.</t>
         </is>
@@ -1222,12 +2103,12 @@
           <t>朝・筋トレ・作業開始</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="M9" s="11" t="inlineStr">
         <is>
           <t>Japanese boom bap with work song energy, heavy taiko kicks, shamisen riffs, shakuhachi, punchy bass, sunrise harbor vibe, 94 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="N9" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A crew of chibi fishermen in indigo hanten and vermilion headbands pulling a net together on a small wooden boat at a sunrise harbor.</t>
         </is>
@@ -1307,12 +2188,12 @@
           <t>瞑想・集中</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="M10" s="11" t="inlineStr">
         <is>
           <t>minimal Japanese lo-fi boom bap, mokugyo wooden block as percussion, singing bowl bell, shakuhachi, deep warm bass, meditative focus, 86 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N10" s="3" t="inlineStr">
+      <c r="N10" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A cheerful chibi monk in a black robe and mustard kesa tapping a wooden mokugyo like a drum, inside a mountain temple hall with incense smoke.</t>
         </is>
@@ -1392,12 +2273,12 @@
           <t>睡眠・休憩</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="M11" s="11" t="inlineStr">
         <is>
           <t>sleepy Japanese chillhop, soft koto, warm electric piano, gentle tape hiss, slow lazy drums, spring nap mood, 68 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N11" s="3" t="inlineStr">
+      <c r="N11" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A little novice monk boy napping on a temple porch with a broom beside him and a cat curled up on his lap, cherry blossom petals drifting.</t>
         </is>
@@ -1477,12 +2358,12 @@
           <t>夜・深夜作業</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M12" s="11" t="inlineStr">
         <is>
           <t>late night Japanese lo-fi hip hop, dusty boom bap drums, shakuhachi echo, muted shamisen, deep bass, moonlit rooftop atmosphere, 87 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr">
+      <c r="N12" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A ninja in an indigo outfit and vermilion scarf sitting on a tiled rooftop at night wearing big headphones, bobbing his head, castle silhouette and full moon in the distance.</t>
         </is>
@@ -1562,12 +2443,12 @@
           <t>勉強・宿題</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="M13" s="11" t="inlineStr">
         <is>
           <t>playful Japanese jazzhop, shinobue flute melody, koto plucks, bouncy swung drums, warm bass, bamboo forest breeze, 90 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N13" s="3" t="inlineStr">
+      <c r="N13" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A clumsy apprentice ninja in a matcha green outfit with an oversized hood balancing on a bamboo stalk in a bamboo forest, determined face.</t>
         </is>
@@ -1647,12 +2528,12 @@
           <t>朝・やる気</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="M14" s="11" t="inlineStr">
         <is>
           <t>energetic Japanese boom bap funk, hyoshigi wooden clappers, taiko, shamisen riffs, punchy bass, brave Edo spirit, 98 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="N14" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. An Edo firefighter in an indigo sashiko hanten twirling a matoi standard in a winter Edo town street with a wooden ladder.</t>
         </is>
@@ -1732,12 +2613,12 @@
           <t>筋トレ・気合い</t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="M15" s="11" t="inlineStr">
         <is>
           <t>hard-hitting Japanese boom bap, massive taiko drums, shime-daiko rolls, shakuhachi, thick bass, bold but friendly groove, 92 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N15" s="3" t="inlineStr">
+      <c r="N15" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A friendly chubby oni with vermilion skin and small horns, mustard waist cloth and indigo headband, joyfully hitting a big taiko drum on a mountain festival tower.</t>
         </is>
@@ -1817,12 +2698,12 @@
           <t>夜・作業・雨の日</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="M16" s="11" t="inlineStr">
         <is>
           <t>late night Japanese jazzhop, rhodes piano, gentle shamisen, upright bass, rain ambience, warm steam and red lantern mood, 80 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N16" s="3" t="inlineStr">
+      <c r="N16" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A quiet ramen stall master in a white samue and indigo apron draining noodles at a small yatai at night after rain, red paper lantern glowing, steam rising.</t>
         </is>
@@ -1902,12 +2783,12 @@
           <t>正月・朝</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="M17" s="11" t="inlineStr">
         <is>
           <t>festive Japanese jazz-funk groove, shinobue flute, kane bells, shime-daiko, electric piano, lucky new year mood, 100 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N17" s="3" t="inlineStr">
+      <c r="N17" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A cute shishimai lion dancer with a vermilion lion head and indigo arabesque body cloth, snapping its jaws playfully in front of a gate with new year pine decorations.</t>
         </is>
@@ -1987,12 +2868,12 @@
           <t>朝・瞑想</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="M18" s="11" t="inlineStr">
         <is>
           <t>airy Japanese ambient hip hop, breathy shakuhachi, soft koto, mountain wind textures, laid-back drums, 82 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N18" s="3" t="inlineStr">
+      <c r="N18" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A wise tengu with a red face and long nose in indigo yamabushi robes, fanning a feather fan on a mountain peak above a sea of clouds with giant cedar trees.</t>
         </is>
@@ -2072,12 +2953,12 @@
           <t>雨の日・夕方</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="M19" s="11" t="inlineStr">
         <is>
           <t>dreamy Japanese jazzhop, koto, shinobue, soft rhodes, sun shower rain sounds, mysterious yet gentle, 76 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N19" s="3" t="inlineStr">
+      <c r="N19" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A quiet procession of chibi foxes in white and indigo kimono holding vermilion umbrellas and lanterns, walking along a rice field path during a sunny rain shower.</t>
         </is>
@@ -2157,12 +3038,12 @@
           <t>夜・考え事</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="M20" s="11" t="inlineStr">
         <is>
           <t>mystical Japanese lo-fi jazzhop, koto, ryuteki flute, deep pads, soft boom bap drums, starry night mood, 83 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N20" s="3" t="inlineStr">
+      <c r="N20" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A cool onmyoji in a white kariginu and indigo trousers with a small floating light at his fingertips in a moonlit garden under a starry sky.</t>
         </is>
@@ -2242,12 +3123,12 @@
           <t>朝・作業</t>
         </is>
       </c>
-      <c r="M21" s="3" t="inlineStr">
+      <c r="M21" s="11" t="inlineStr">
         <is>
           <t>serene Japanese jazzhop, kagura bells, koto, shinobue, soft electric piano, crisp autumn morning, 80 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N21" s="3" t="inlineStr">
+      <c r="N21" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A shrine maiden in white kimono and vermilion hakama sweeping fallen maple leaves with a bamboo broom in a quiet shrine courtyard in the morning, torii gate behind.</t>
         </is>
@@ -2327,12 +3208,12 @@
           <t>朝・お出かけ</t>
         </is>
       </c>
-      <c r="M22" s="3" t="inlineStr">
+      <c r="M22" s="11" t="inlineStr">
         <is>
           <t>gentle festive Japanese jazzhop, small bells, shinobue, tsuzumi, warm bass, innocent cheerful mood, 90 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N22" s="3" t="inlineStr">
+      <c r="N22" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A small festival child in a vermilion and gold ceremonial costume with a tiny crown, shaking a bell shyly on top of a festival float.</t>
         </is>
@@ -2412,12 +3293,12 @@
           <t>昼・リラックス</t>
         </is>
       </c>
-      <c r="M23" s="3" t="inlineStr">
+      <c r="M23" s="11" t="inlineStr">
         <is>
           <t>elegant Japanese bossa jazzhop, koto, sho mouth organ pads, nylon guitar, rhodes, light swing drums, graceful spring garden, 86 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N23" s="3" t="inlineStr">
+      <c r="N23" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A Heian noble in an indigo nōshi robe and black eboshi hat gracefully kicking a kemari ball in a spring garden under wisteria.</t>
         </is>
@@ -2497,12 +3378,12 @@
           <t>気合い・作業</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="M24" s="11" t="inlineStr">
         <is>
           <t>dramatic yet groovy Japanese boom bap, hyoshigi clappers, shamisen riffs, tsuzumi, punchy drums, theatrical energy, 93 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N24" s="3" t="inlineStr">
+      <c r="N24" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A kabuki actor with vermilion and indigo kumadori makeup in a mustard costume striking a mie pose on a wooden theater stage lined with lanterns.</t>
         </is>
@@ -2582,12 +3463,12 @@
           <t>集中・筋トレ</t>
         </is>
       </c>
-      <c r="M25" s="3" t="inlineStr">
+      <c r="M25" s="11" t="inlineStr">
         <is>
           <t>powerful Japanese boom bap, deep taiko, subtle conch horn texture, shakuhachi, heavy bass, steady disciplined groove, 88 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N25" s="3" t="inlineStr">
+      <c r="N25" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A big friendly warrior monk with a white hood and black robe holding a conch shell, standing in front of a temple gate on stone steps.</t>
         </is>
@@ -2667,12 +3548,12 @@
           <t>昼・リラックス</t>
         </is>
       </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="M26" s="11" t="inlineStr">
         <is>
           <t>laid-back Japanese jazzhop, upright bass lead, koto, electric piano, river water ambience, summer shade mood, 84 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N26" s="3" t="inlineStr">
+      <c r="N26" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A cute kappa with matcha green skin and an indigo bib plucking an upright bass on a riverbank under a willow tree, cucumber beside him.</t>
         </is>
@@ -2752,12 +3633,12 @@
           <t>夕方・買い物気分</t>
         </is>
       </c>
-      <c r="M27" s="3" t="inlineStr">
+      <c r="M27" s="11" t="inlineStr">
         <is>
           <t>warm Japanese city groove, electric piano, funky bass, little bells, shamisen accents, nostalgic shopping street at dusk, 95 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N27" s="3" t="inlineStr">
+      <c r="N27" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A maneki-neko lucky cat with a vermilion collar and mustard bell beckoning with its paw in front of a small shop on a nostalgic shopping street at dusk.</t>
         </is>
@@ -2837,12 +3718,12 @@
           <t>夜・読書</t>
         </is>
       </c>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="M28" s="11" t="inlineStr">
         <is>
           <t>moody Japanese jazzhop boom bap, biwa lute riffs, shakuhachi, warm bass, dusty drums, storytelling autumn mood, 82 bpm, instrumental, no vocals</t>
         </is>
       </c>
-      <c r="N28" s="3" t="inlineStr">
+      <c r="N28" s="12" t="inlineStr">
         <is>
           <t>Chibi character with 2 to 2.5 head-tall proportions, thick bold outlines, slightly retro 1980s-90s Japanese anime style, flat cel shading with soft film grain, muted traditional Japanese color palette of indigo, vermilion, mustard yellow and matcha green on a warm washi-paper toned background, cozy and wholesome mood, simple readable shapes, single still illustration in 16:9, no text, no logo. A traveling biwa player monk in dark robes and mustard hood strumming a biwa at a mountain teahouse in autumn, falling leaves.</t>
         </is>
@@ -2869,7 +3750,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3212,7 +4093,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3266,7 +4147,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>タイトル案</t>
+          <t>【YouTube】動画タイトル（コピペ）</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -3279,9 +4160,9 @@
           <t>サムネ案</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>サムネ用プロンプト（英語）</t>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>【ChatGPT】サムネ画像プロンプト（コピペ）</t>
         </is>
       </c>
     </row>
@@ -3329,7 +4210,7 @@
           <t>師弟の後ろ姿／満月／「深夜」</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi ninjas on a moonlit tiled rooftop: the rooftop ninja in indigo with a vermilion scarf wearing big headphones, the small apprentice ninja in matcha green holding a scroll, one ninja playing a shakuhachi, one tapping a small taiko drum, one spinning a vinyl record, one jumping high over a hemp plant. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
@@ -3379,7 +4260,7 @@
           <t>隊長と若侍／夕焼けの城／「集中」</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J3" s="12" t="inlineStr">
         <is>
           <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi samurai jumping on stone steps of a castle town at sunset: the captain in an indigo haori with big headphones, the young samurai hugging a vinyl record, one holding a big rice ball, one beating a small taiko drum, one playing a shakuhachi, one waving a folding fan. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
@@ -3429,7 +4310,7 @@
           <t>縁側とスイカ／河童／「夏休み」</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="12" t="inlineStr">
         <is>
           <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: five chibi characters splashing at a summer riverside: the off-duty samurai in an indigo yukata waving an uchiwa fan, the kappa plucking an upright bass, one holding a slice of watermelon, one ringing a wind chime, one jumping with a cucumber, plus a friend with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
@@ -3479,7 +4360,7 @@
           <t>赤提灯／湯気／浪人の編笠</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters around a ramen stall at night after rain: the stall master tossing noodles with a strainer, the ronin DJ in a straw hat scratching a turntable, one slurping noodles, one playing a shamisen, one dancing with a paper umbrella, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
@@ -3529,7 +4410,7 @@
           <t>木魚／眠る小僧と猫／桜</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: five chibi characters bouncing in a spring temple hall with cherry blossoms: the cheerful monk tapping a mokugyo, the novice monk boy hopping with a broom, a cat jumping, one monk ringing a small bell, one wearing big headphones and dancing. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
@@ -3579,7 +4460,7 @@
           <t>踊る連／太鼓の鬼／提灯</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J7" s="12" t="inlineStr">
         <is>
           <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi festival dancers on a lantern-lit street: the friendly oni beating a big taiko drum, Awa-odori dancers in indigo happi coats raising their hands, one waving an uchiwa fan, one ringing a kane bell, one playing a shinobue flute, one jumping with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
@@ -3629,7 +4510,7 @@
           <t>狐の行列／鳥居／和傘</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters in a shrine courtyard during a sun shower: the shrine maiden in vermilion hakama shaking kagura bells, a fox bride in white holding a vermilion umbrella, fox friends hopping with paper lanterns, one fox playing a shinobue flute, one twirling an umbrella, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
@@ -3679,7 +4560,7 @@
           <t>蹴鞠／藤棚／星空</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J9" s="12" t="inlineStr">
         <is>
           <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi Heian characters in a spring garden under wisteria: a noble in an indigo robe kicking a kemari ball high, the onmyoji with a small floating light, the festival child shaking a bell, one playing a koto, one dancing with a folding fan, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
@@ -3729,7 +4610,7 @@
           <t>獅子舞／若殿／「福」</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters at a New Year gate with pine decorations: the shishimai lion dancer snapping its jaws, the young lord in a vermilion kamishimo jumping, the maneki-neko cat beckoning, one retainer beating a small taiko drum, one playing a shinobue flute, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
@@ -3779,7 +4660,7 @@
           <t>三味線／隈取／提灯</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi performers on a wooden theater stage lined with lanterns: the kabuki actor with kumadori makeup striking a pose, an elegant musician lady in modest fully covered kimono playing a shamisen, the biwa player strumming, one clapping hyoshigi wooden clappers, one beating a small taiko drum, one jumping with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
         </is>
@@ -3791,7 +4672,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3817,9 +4698,9 @@
           <t>企画No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>曲タイトル</t>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>【Suno】Title欄（曲タイトル）</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -3842,14 +4723,14 @@
           <t>BPM</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Suno スタイル（英語）</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>歌詞（Suno Lyrics欄に貼る）</t>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>【Suno】Style欄にコピペ</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>【Suno】Lyrics欄にコピペ</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -3862,7 +4743,7 @@
       <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>麻とびこえて、きょうもワンステップ</t>
         </is>
@@ -3885,12 +4766,12 @@
       <c r="F2" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>Japanese jazzy hip hop, upbeat groove, 100 BPM, punchy boom bap drums, funky bassline, Japanese shakuhachi, Japanese shamisen, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>[Verse]
 やねのうえ　つきが　まるい
@@ -3926,7 +4807,7 @@
       <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>腹が減っては、ビートはできぬ</t>
         </is>
@@ -3949,12 +4830,12 @@
       <c r="F3" s="3" t="n">
         <v>96</v>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>Japanese jazzy hip hop, upbeat groove, 96 BPM, punchy boom bap drums, funky bassline, Japanese shamisen, Japanese shakuhachi, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>[Verse]
 いしだんに　ならんで　すわる
@@ -3988,7 +4869,7 @@
       <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>鬼に金棒、河童にベース</t>
         </is>
@@ -4011,12 +4892,12 @@
       <c r="F4" s="3" t="n">
         <v>98</v>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>Japanese jazzy hip hop, upbeat groove, 98 BPM, punchy boom bap drums, funky bassline, Japanese koto, Japanese shamisen, bright female vocal, Japanese lyrics, energetic, bright, head nod</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>[Verse]
 えんがわで　うちわを　ぱたぱた
@@ -4050,7 +4931,7 @@
       <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>二八そばより、十六ビート</t>
         </is>
@@ -4073,12 +4954,12 @@
       <c r="F5" s="3" t="n">
         <v>100</v>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>Japanese jazzy hip hop, upbeat groove, 100 BPM, punchy boom bap drums, funky bassline, Japanese shamisen, Japanese shakuhachi, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>[Verse]
 あめあがり　あかちょうちん
@@ -4112,7 +4993,7 @@
       <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>魚は眠らず、小僧は眠る</t>
         </is>
@@ -4135,12 +5016,12 @@
       <c r="F6" s="3" t="n">
         <v>96</v>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>Japanese jazzy hip hop, upbeat groove, 96 BPM, punchy boom bap drums, funky bassline, Japanese shakuhachi, Japanese koto, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>[Verse]
 ぽく　ぽく　ぽく　と　ほんどうに
@@ -4174,7 +5055,7 @@
       <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>踊る阿呆に、太鼓たたく鬼</t>
         </is>
@@ -4197,12 +5078,12 @@
       <c r="F7" s="3" t="n">
         <v>104</v>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>Japanese jazzy hip hop, upbeat groove, 104 BPM, punchy boom bap drums, funky bassline, Japanese shinobue, Japanese shamisen, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>[Verse]
 ちょうちんの　あかりが　つづく　みち
@@ -4236,7 +5117,7 @@
       <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>お天気雨は、狐の招待状</t>
         </is>
@@ -4259,12 +5140,12 @@
       <c r="F8" s="3" t="n">
         <v>96</v>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>Japanese jazzy hip hop, upbeat groove, 96 BPM, punchy boom bap drums, funky bassline, Japanese koto, Japanese shinobue, bright female vocal, Japanese lyrics, energetic, bright, head nod</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>[Verse]
 はれているのに　ぽつ　ぽつ　ぽつ
@@ -4298,7 +5179,7 @@
       <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>いとをかし、いとグルーヴィ</t>
         </is>
@@ -4321,12 +5202,12 @@
       <c r="F9" s="3" t="n">
         <v>98</v>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>Japanese jazzy hip hop, upbeat groove, 98 BPM, punchy boom bap drums, funky bassline, Japanese koto, Japanese ryuteki flute, bright female vocal, Japanese lyrics, energetic, bright, head nod</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="11" t="inlineStr">
         <is>
           <t>[Verse]
 ふじの　はなが　ゆれる　にわ
@@ -4360,7 +5241,7 @@
       <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>猫の手も、招きたいお正月</t>
         </is>
@@ -4383,12 +5264,12 @@
       <c r="F10" s="3" t="n">
         <v>102</v>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>Japanese jazzy hip hop, upbeat groove, 102 BPM, punchy boom bap drums, funky bassline, Japanese shinobue, Japanese shamisen, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>[Verse]
 おしょうがつ　まつかざりの　もん
@@ -4422,7 +5303,7 @@
       <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>待ってました、と言わせたい</t>
         </is>
@@ -4445,12 +5326,12 @@
       <c r="F11" s="3" t="n">
         <v>98</v>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>Japanese jazzy hip hop, upbeat groove, 98 BPM, punchy boom bap drums, funky bassline, Japanese shamisen, Japanese biwa, taiko drums, energetic male vocal, Japanese lyrics, energetic, bright, head nod</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>[Verse]
 ひょうしぎ　かん　かん　まくが　あく

</xml_diff>

<commit_message>
Switch thumbnail prompts to straight-row lineup on solid backgrounds for animation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S9ZzjqDoB7HA6WESKfKq7k
</commit_message>
<xml_diff>
--- a/wa_groove企画/wa_groove_characters.xlsx
+++ b/wa_groove企画/wa_groove_characters.xlsx
@@ -778,7 +778,7 @@
       </c>
       <c r="F1" s="10" t="inlineStr">
         <is>
-          <t>④ 【ChatGPT】サムネ画像</t>
+          <t>④ 【ChatGPT】並び絵プロンプト（サムネ・アニメ共通）</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="F2" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi ninjas on a moonlit tiled rooftop: the rooftop ninja in indigo with a vermilion scarf wearing big headphones, the small apprentice ninja in matcha green holding a scroll, one ninja playing a shakuhachi, one tapping a small taiko drum, one spinning a vinyl record, one jumping high over a hemp plant. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: a ninja in a brown outfit holding a shakuhachi, the small apprentice ninja in matcha green holding a scroll, the rooftop ninja in indigo with a vermilion scarf wearing big headphones, a ninja in vermilion holding a small taiko drum, a ninja in purple holding a vinyl record, a ninja in charcoal gray holding a folding fan. Plain solid mustard yellow background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="F3" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi samurai jumping on stone steps of a castle town at sunset: the captain in an indigo haori with big headphones, the young samurai hugging a vinyl record, one holding a big rice ball, one beating a small taiko drum, one playing a shakuhachi, one waving a folding fan. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the samurai captain in an indigo haori with arms crossed and headphones around his neck, the young samurai hugging a vinyl record, a samurai holding a big rice ball, a samurai holding a small taiko drum, a samurai holding a shakuhachi, a samurai holding a folding fan. Plain solid matcha green background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="F4" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: five chibi characters splashing at a summer riverside: the off-duty samurai in an indigo yukata waving an uchiwa fan, the kappa plucking an upright bass, one holding a slice of watermelon, one ringing a wind chime, one jumping with a cucumber, plus a friend with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the off-duty samurai in a white yukata holding an uchiwa fan, the kappa holding an upright bass, a child holding a slice of watermelon, a girl in a yukata holding a wind chime, a samurai holding a cucumber, a friend wearing big headphones holding a pinwheel. Plain solid soft indigo blue background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters around a ramen stall at night after rain: the stall master tossing noodles with a strainer, the ronin DJ in a straw hat scratching a turntable, one slurping noodles, one playing a shamisen, one dancing with a paper umbrella, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the ramen stall master in a white samue holding a noodle strainer, the ronin in a woven straw hat holding a vinyl record, a customer holding a ramen bowl, a musician holding a shamisen, a girl holding a paper umbrella, a boy holding a red paper lantern. Plain solid deep indigo background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: five chibi characters bouncing in a spring temple hall with cherry blossoms: the cheerful monk tapping a mokugyo, the novice monk boy hopping with a broom, a cat jumping, one monk ringing a small bell, one wearing big headphones and dancing. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the cheerful monk holding a mokugyo, the novice monk boy holding a broom, a small cat sitting upright, a monk holding a small bell, a novice holding a teacup, a monk wearing big headphones. Plain solid pale cherry blossom pink background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi festival dancers on a lantern-lit street: the friendly oni beating a big taiko drum, Awa-odori dancers in indigo happi coats raising their hands, one waving an uchiwa fan, one ringing a kane bell, one playing a shinobue flute, one jumping with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the friendly oni with vermilion skin holding a taiko drum, an Awa-odori dancer in an indigo happi coat holding an uchiwa fan, a dancer holding a kane bell, a dancer playing a shinobue flute, a female dancer in a straw hat with raised hands, a dancer holding a paper lantern. Plain solid mustard yellow background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters in a shrine courtyard during a sun shower: the shrine maiden in vermilion hakama shaking kagura bells, a fox bride in white holding a vermilion umbrella, fox friends hopping with paper lanterns, one fox playing a shinobue flute, one twirling an umbrella, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the shrine maiden in vermilion hakama holding kagura bells, a fox bride in white holding a vermilion umbrella, a fox holding a paper lantern, a fox holding a shinobue flute, a fox holding a small umbrella, a fox wearing big headphones. Plain solid matcha green background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi Heian characters in a spring garden under wisteria: a noble in an indigo robe kicking a kemari ball high, the onmyoji with a small floating light, the festival child shaking a bell, one playing a koto, one dancing with a folding fan, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: a Heian noble in an indigo robe holding a kemari ball, the onmyoji in white with a small floating light above his hand, the festival child holding a bell, a court lady holding a folding fan, a musician holding a ryuteki flute, a noble holding a tsuzumi hand drum. Plain solid soft indigo blue background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters at a New Year gate with pine decorations: the shishimai lion dancer snapping its jaws, the young lord in a vermilion kamishimo jumping, the maneki-neko cat beckoning, one retainer beating a small taiko drum, one playing a shinobue flute, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the shishimai lion dancer with a red lion head, the young lord in a gold kamishimo, the maneki-neko cat beckoning with one paw, a retainer in indigo holding a small taiko drum, a retainer holding a shinobue flute, a retainer holding a New Year kite. Plain solid vermilion red background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi performers on a wooden theater stage lined with lanterns: the kabuki actor with kumadori makeup striking a pose, an elegant musician lady in modest fully covered kimono playing a shamisen, the biwa player strumming, one clapping hyoshigi wooden clappers, one beating a small taiko drum, one jumping with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the kabuki actor with kumadori makeup holding a folding fan, an elegant musician lady in a modest fully covered kimono holding a shamisen, the biwa player holding a biwa, a stagehand holding hyoshigi wooden clappers, a drummer holding a small taiko drum, a fan waving a paper lantern. Plain solid deep indigo background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -3756,7 +3756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4084,6 +4084,91 @@
       <c r="C19" s="3" t="inlineStr">
         <is>
           <t>laid back, mellow, night, calm（※上の「避けるタグ（歌入り誘発）」はインスト版用）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>アニメ用の並び絵</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>1. 横一列・重ならない</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>キャラ同士の間をあけて横一列に。重なっていないと「背景を削除」やCanvaで1人ずつ切り抜いて動かせる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>アニメ用の並び絵</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>2. 足元の高さをそろえる</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>全員の足を同じ高さ（同じ線）に置く。頭の上下やジャンプのループを付けてもズレが目立たない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>アニメ用の並び絵</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>3. 背景は単色</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>背景が1色なら切り抜きがきれいに抜ける。回ごとに背景色だけ変えるとシリーズ感が出る。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>アニメ用の並び絵</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>4. 上の1/3は空ける</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>タイトル文字はCanvaで上の空きスペースに後から入れる。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>アニメ用の並び絵</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>5. 簡単な動きの例</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>頭を上下にゆらす／体を左右にゆらす／小さくジャンプ／持ち物（太鼓のバチ・うちわ）だけ動かす。1人ずつタイミングをずらすと生き生きする。</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4247,7 @@
       </c>
       <c r="J1" s="10" t="inlineStr">
         <is>
-          <t>【ChatGPT】サムネ画像プロンプト（コピペ）</t>
+          <t>【ChatGPT】並び絵プロンプト（サムネ・アニメ共通）</t>
         </is>
       </c>
     </row>
@@ -4212,7 +4297,7 @@
       </c>
       <c r="J2" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi ninjas on a moonlit tiled rooftop: the rooftop ninja in indigo with a vermilion scarf wearing big headphones, the small apprentice ninja in matcha green holding a scroll, one ninja playing a shakuhachi, one tapping a small taiko drum, one spinning a vinyl record, one jumping high over a hemp plant. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: a ninja in a brown outfit holding a shakuhachi, the small apprentice ninja in matcha green holding a scroll, the rooftop ninja in indigo with a vermilion scarf wearing big headphones, a ninja in vermilion holding a small taiko drum, a ninja in purple holding a vinyl record, a ninja in charcoal gray holding a folding fan. Plain solid mustard yellow background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -4262,7 +4347,7 @@
       </c>
       <c r="J3" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi samurai jumping on stone steps of a castle town at sunset: the captain in an indigo haori with big headphones, the young samurai hugging a vinyl record, one holding a big rice ball, one beating a small taiko drum, one playing a shakuhachi, one waving a folding fan. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the samurai captain in an indigo haori with arms crossed and headphones around his neck, the young samurai hugging a vinyl record, a samurai holding a big rice ball, a samurai holding a small taiko drum, a samurai holding a shakuhachi, a samurai holding a folding fan. Plain solid matcha green background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -4312,7 +4397,7 @@
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: five chibi characters splashing at a summer riverside: the off-duty samurai in an indigo yukata waving an uchiwa fan, the kappa plucking an upright bass, one holding a slice of watermelon, one ringing a wind chime, one jumping with a cucumber, plus a friend with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the off-duty samurai in a white yukata holding an uchiwa fan, the kappa holding an upright bass, a child holding a slice of watermelon, a girl in a yukata holding a wind chime, a samurai holding a cucumber, a friend wearing big headphones holding a pinwheel. Plain solid soft indigo blue background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -4362,7 +4447,7 @@
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters around a ramen stall at night after rain: the stall master tossing noodles with a strainer, the ronin DJ in a straw hat scratching a turntable, one slurping noodles, one playing a shamisen, one dancing with a paper umbrella, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the ramen stall master in a white samue holding a noodle strainer, the ronin in a woven straw hat holding a vinyl record, a customer holding a ramen bowl, a musician holding a shamisen, a girl holding a paper umbrella, a boy holding a red paper lantern. Plain solid deep indigo background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -4412,7 +4497,7 @@
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: five chibi characters bouncing in a spring temple hall with cherry blossoms: the cheerful monk tapping a mokugyo, the novice monk boy hopping with a broom, a cat jumping, one monk ringing a small bell, one wearing big headphones and dancing. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the cheerful monk holding a mokugyo, the novice monk boy holding a broom, a small cat sitting upright, a monk holding a small bell, a novice holding a teacup, a monk wearing big headphones. Plain solid pale cherry blossom pink background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4547,7 @@
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi festival dancers on a lantern-lit street: the friendly oni beating a big taiko drum, Awa-odori dancers in indigo happi coats raising their hands, one waving an uchiwa fan, one ringing a kane bell, one playing a shinobue flute, one jumping with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the friendly oni with vermilion skin holding a taiko drum, an Awa-odori dancer in an indigo happi coat holding an uchiwa fan, a dancer holding a kane bell, a dancer playing a shinobue flute, a female dancer in a straw hat with raised hands, a dancer holding a paper lantern. Plain solid mustard yellow background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -4512,7 +4597,7 @@
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters in a shrine courtyard during a sun shower: the shrine maiden in vermilion hakama shaking kagura bells, a fox bride in white holding a vermilion umbrella, fox friends hopping with paper lanterns, one fox playing a shinobue flute, one twirling an umbrella, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the shrine maiden in vermilion hakama holding kagura bells, a fox bride in white holding a vermilion umbrella, a fox holding a paper lantern, a fox holding a shinobue flute, a fox holding a small umbrella, a fox wearing big headphones. Plain solid matcha green background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -4562,7 +4647,7 @@
       </c>
       <c r="J9" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi Heian characters in a spring garden under wisteria: a noble in an indigo robe kicking a kemari ball high, the onmyoji with a small floating light, the festival child shaking a bell, one playing a koto, one dancing with a folding fan, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: a Heian noble in an indigo robe holding a kemari ball, the onmyoji in white with a small floating light above his hand, the festival child holding a bell, a court lady holding a folding fan, a musician holding a ryuteki flute, a noble holding a tsuzumi hand drum. Plain solid soft indigo blue background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -4612,7 +4697,7 @@
       </c>
       <c r="J10" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi characters at a New Year gate with pine decorations: the shishimai lion dancer snapping its jaws, the young lord in a vermilion kamishimo jumping, the maneki-neko cat beckoning, one retainer beating a small taiko drum, one playing a shinobue flute, one wearing big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the shishimai lion dancer with a red lion head, the young lord in a gold kamishimo, the maneki-neko cat beckoning with one paw, a retainer in indigo holding a small taiko drum, a retainer holding a shinobue flute, a retainer holding a New Year kite. Plain solid vermilion red background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>
@@ -4662,7 +4747,7 @@
       </c>
       <c r="J11" s="12" t="inlineStr">
         <is>
-          <t>YouTube thumbnail illustration, 16:9. cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. The character group is the main subject: six chibi performers on a wooden theater stage lined with lanterns: the kabuki actor with kumadori makeup striking a pose, an elegant musician lady in modest fully covered kimono playing a shamisen, the biwa player strumming, one clapping hyoshigi wooden clappers, one beating a small taiko drum, one jumping with big headphones. All of them face the viewer with lively jumping and dancing poses, each holding a different prop. Leave clear empty space in the upper-left corner for text. Lively, playful, energetic. No text, no letters, no logos, no watermark.</t>
+          <t>cute chibi characters (2–2.5 heads tall), thick clean outlines, slightly retro Japanese anime look, muted traditional Japanese colors (indigo, vermilion, mustard yellow, matcha green), soft grain texture. Six chibi characters standing side by side in one straight horizontal row, evenly spaced with clear gaps so no one overlaps, similar height, full body from head to feet, feet on the same baseline, all facing the viewer, simple relaxed standing pose, each holding a different prop. From left to right: the kabuki actor with kumadori makeup holding a folding fan, an elegant musician lady in a modest fully covered kimono holding a shamisen, the biwa player holding a biwa, a stagehand holding hyoshigi wooden clappers, a drummer holding a small taiko drum, a fan waving a paper lantern. Plain solid deep indigo background, no scenery, no floor, no cast shadows. Characters in the lower two-thirds of the image, leave the top third empty for title text. 16:9. Cheerful and playful. No text, no letters, no logos, no watermark.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add dance pose frame prompts sheet for simple loop animation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S9ZzjqDoB7HA6WESKfKq7k
</commit_message>
<xml_diff>
--- a/wa_groove企画/wa_groove_characters.xlsx
+++ b/wa_groove企画/wa_groove_characters.xlsx
@@ -9,16 +9,17 @@
   <sheets>
     <sheet name="使い方" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="コピペ早見表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="キャラ一覧" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="共通スタイル" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="動画企画案" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="歌詞" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ダンス差分" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="キャラ一覧" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="共通スタイル" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="動画企画案" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="歌詞" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'キャラ一覧'!$A$1:$Q$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'共通スタイル'!$A$1:$C$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'動画企画案'!$A$1:$J$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'歌詞'!$A$1:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'キャラ一覧'!$A$1:$Q$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'共通スタイル'!$A$1:$C$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'動画企画案'!$A$1:$J$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'歌詞'!$A$1:$I$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -126,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -163,6 +164,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -530,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -723,6 +730,23 @@
       <c r="A30" s="5" t="inlineStr">
         <is>
           <t>→ Googleスプレッドシートで見る場合は、このxlsxをGoogleドライブにアップして開くとシートの切り替えもそのまま使えます。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>並び絵を踊らせる（ダンス差分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>「ダンス差分」シートのプロンプトで、同じ並び絵のポーズ違いを4枚作り、パラパラ切り替えて踊っているように見せます</t>
         </is>
       </c>
     </row>
@@ -1335,6 +1359,248 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="100" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>コマ</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>コマ名</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>使いどころ</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>表示時間の目安（BPM100なら1拍＝0.6秒）</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>【ChatGPT】差分プロンプト（並び絵を添付してコピペ）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>基本（もとの並び絵）</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>今ある並び絵をそのまま使う。プロンプト不要</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>1拍</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>ゆれ右（交互）</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Aと交互に表示してノリを出す基本の動き</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>1拍</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Edit the attached image. Keep everything exactly the same: the same six characters, same art style, same colors, same outfits, same props, same plain solid background, same size, same left-to-right order and positions, same framing. Only change the poses: a fun dance move. Counting from the left, characters 1, 3 and 5 lean their bodies to the right and lift their left foot slightly; characters 2, 4 and 6 lean to the left and lift their right foot slightly. Heads tilt with the lean, happy smiling faces, props raised a little. Feet stay close to the same baseline. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>ゆれ左（交互）</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Bの左右反対。A→B→A→C でくり返すと踊って見える</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>1拍</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Edit the attached image. Keep everything exactly the same: the same six characters, same art style, same colors, same outfits, same props, same plain solid background, same size, same left-to-right order and positions, same framing. Only change the poses: a fun dance move, mirrored from the previous pose. Counting from the left, characters 1, 3 and 5 lean their bodies to the left and lift their right foot slightly; characters 2, 4 and 6 lean to the right and lift their left foot slightly. Heads tilt with the lean, happy smiling faces, props raised a little. Feet stay close to the same baseline. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>うなずき（ヘッドノッド）</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ビートに合わせたうなずき。Aと交互にすると落ち着いたノリ</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>半拍</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Edit the attached image. Keep everything exactly the same: the same six characters, same art style, same colors, same outfits, same props, same plain solid background, same size, same left-to-right order and positions, same framing. Only change the poses: a head-nod groove. All six characters bend their knees slightly and dip their heads down, eyes closed with content smiles, as if nodding to the beat. Bodies stay in place. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>ジャンプ（サビ用）</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>サビや盛り上がりで数回だけ入れる決めポーズ</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>1拍</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Edit the attached image. Keep everything exactly the same: the same six characters, same art style, same colors, same outfits, same props, same plain solid background, same size, same left-to-right order and positions, same framing. Only change the poses: a joyful jump. All six characters jump slightly with both arms raised, holding their props up high, feet just off the ground, big open-mouth smiles. Keep the same horizontal positions. No text, no letters, no logos, no watermark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>作り方</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>1. 並び絵（コマA）ができたチャットで、その画像を添付したまま B→C→D→E の順にプロンプトを1つずつ送る（1回に1枚）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2. キャラの位置や服がズレたら「↻」で作り直す。ズレが大きいときは、コマAを添付し直して新しいチャットで送る</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>3. 全コマを同じ名前ルールで保存（例：01_A.png, 01_B.png …　01は企画No）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>4. CapCut／Canvaで A→B→A→C を1拍ずつ並べてループ。サビで E をはさむ。うなずきだけにしたいときは A→D をくり返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>5. 曲のBPMに合わせると気持ちよく見える：BPM96＝0.63秒、BPM100＝0.6秒、BPM104＝0.58秒（60÷BPM）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>コツ：B・Cは奇数番目と偶数番目が逆に動くので、2枚だけでも「波」のように踊って見えます</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A10:E10"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A9:E9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3750,7 +4016,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4178,7 +4444,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4757,7 +5023,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add 8-track ninja series sheet with Suno prompts, lyrics and auto timestamps
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01S9ZzjqDoB7HA6WESKfKq7k
</commit_message>
<xml_diff>
--- a/wa_groove企画/wa_groove_characters.xlsx
+++ b/wa_groove企画/wa_groove_characters.xlsx
@@ -9,17 +9,18 @@
   <sheets>
     <sheet name="使い方" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="コピペ早見表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ダンス差分" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="キャラ一覧" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="共通スタイル" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="動画企画案" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="歌詞" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="忍者シリーズ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ダンス差分" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="キャラ一覧" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="共通スタイル" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="動画企画案" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="歌詞" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'キャラ一覧'!$A$1:$Q$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'共通スタイル'!$A$1:$C$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'動画企画案'!$A$1:$J$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'歌詞'!$A$1:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'キャラ一覧'!$A$1:$Q$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'共通スタイル'!$A$1:$C$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'動画企画案'!$A$1:$J$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'歌詞'!$A$1:$I$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -28,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,8 +68,13 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +106,11 @@
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -127,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -170,6 +181,13 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -537,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -747,6 +765,23 @@
       <c r="A33" s="13" t="inlineStr">
         <is>
           <t>「ダンス差分」シートのプロンプトで、同じ並び絵のポーズ違いを4枚作り、パラパラ切り替えて踊っているように見せます</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>忍者シリーズ（30分動画・8曲）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>「忍者シリーズ」シートに8曲分のSuno用①〜④と、概要欄のタイムスタンプが自動で作れる欄があります</t>
         </is>
       </c>
     </row>
@@ -1361,6 +1396,852 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C55A11"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="56" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>曲順</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>場面</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>歌／インスト</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>BPM</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>① 【Suno】Title欄</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>元ネタ・洒落のポイント</t>
+        </is>
+      </c>
+      <c r="G1" s="9" t="inlineStr">
+        <is>
+          <t>② 【Suno】Style欄</t>
+        </is>
+      </c>
+      <c r="H1" s="9" t="inlineStr">
+        <is>
+          <t>③ 【Suno】Lyrics欄</t>
+        </is>
+      </c>
+      <c r="I1" s="9" t="inlineStr">
+        <is>
+          <t>④ 【Suno】Exclude Styles欄</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>できた長さ（分）</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>できた長さ（秒）</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>タイムスタンプ</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>⑤ 【YouTube】概要欄トラックリスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>朝｜夜明けの屋根から修行に出発</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>歌</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>早起きは三文の徳、屋根の上なら五文の徳</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>ことわざ「早起きは三文の徳」。屋根の上ならもっと得、という洒落</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>Japanese groove pop, upbeat, bright and refreshing, 100 BPM, punchy drums, funky bassline, Japanese shakuhachi, Japanese shamisen, light taiko drums, sunrise feeling, energetic male vocal, Japanese lyrics, Japanese call-and-response chants, male group chorus, head nod</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
+        <is>
+          <t>[Intro]
+（そーれ）
+[Verse]
+あさひが　かわらを　そめていく
+とりより　はやく　めを　さませ
+ずきんを　きゅっと　むすんだら
+きょうの　しゅぎょうの　はじまりだ
+[Pre-Chorus]
+まちは　まだ　ねむってる
+いまのうちに　かけだそう
+[Chorus]
+はやおき（はっ）　さんもん（それ）　とくを　する
+やねの　うえなら　ごもんの　とく
+とんで　はねて　あさひへ　とどけ
+きょうも　いちばん　のりで　いこう
+[Instrumental Break]
+[Verse]
+みそしる　におう　まちかどを
+かぜより　はやく　すりぬける
+さかなやさんが　てを　ふって
+いってらっしゃいと　わらってる
+[Pre-Chorus]
+まちが　すこし　めを　さます
+いまのうちに　かけだそう
+[Chorus]
+はやおき（はっ）　さんもん（それ）　とくを　する
+やねの　うえなら　ごもんの　とく
+とんで　はねて　あさひへ　とどけ
+きょうも　いちばん　のりで　いこう
+[Bridge]
+いよっ（いよっ）　そーれ（そーれ）
+こえを　あわせて　もういっかい
+[Chorus]
+はやおき（はっ）　さんもん（それ）　とくを　する
+やねの　うえなら　ごもんの　とく
+とんで　はねて　あさひへ　とどけ
+きょうも　いちばん　のりで　いこう
+[Outro]
+（そーれ）</t>
+        </is>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>dark, horror, scary, English lyrics, rap, epic, cinematic</t>
+        </is>
+      </c>
+      <c r="J2" s="15" t="n"/>
+      <c r="K2" s="15" t="n"/>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="M2" s="3">
+        <f>L2&amp;" "&amp;E2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>昼前｜手裏剣の稽古（木の的）</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>歌</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>当たるも八卦、投げるも手裏剣</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ことわざ「当たるも八卦当たらぬも八卦」のもじり</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>Japanese groove pop, upbeat, bright and refreshing, 102 BPM, punchy drums, funky bassline, Japanese shakuhachi, Japanese shamisen riffs, crisp percussion, energetic male vocal, Japanese lyrics, Japanese call-and-response chants, male group chorus, head nod</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>[Intro]
+（えいさ）
+[Verse]
+きの　まとを　ずらりと　ならべ
+ひとつ　ふたつと　かぞえたら
+てくびを　かえして　しゅっと　なげ
+かぜを　きる　おと　ここちいい
+[Pre-Chorus]
+あたるも　はっけ　あたらぬも
+わらって　もう　ひとつ
+[Chorus]
+しゅっ　しゅっ（はっ）　まわれ（それ）　ほしの　かたち
+くるくる　ひかって　まとの　まんなか
+はずれても（よいしょ）　めげないで（それ）
+つぎの　いちまい　いきを　すって
+[Instrumental Break]
+[Verse]
+ししょうの　てほんは　みえないほど
+はやくて　しずかで　うつくしい
+おいらは　まだまだ　みならいだけど
+きのうより　ひとつ　うまくなる
+[Pre-Chorus]
+あたるも　はっけ　あたらぬも
+わらって　もう　ひとつ
+[Chorus]
+しゅっ　しゅっ（はっ）　まわれ（それ）　ほしの　かたち
+くるくる　ひかって　まとの　まんなか
+はずれても（よいしょ）　めげないで（それ）
+つぎの　いちまい　いきを　すって
+[Bridge]
+ひとつ（えいさ）　ふたつ（えいさ）
+みっつ　よっつで　どまんなか
+[Chorus]
+しゅっ　しゅっ（はっ）　まわれ（それ）　ほしの　かたち
+くるくる　ひかって　まとの　まんなか
+はずれても（よいしょ）　めげないで（それ）
+つぎの　いちまい　いきを　すって
+[Outro]
+（えいさ）</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>dark, horror, scary, English lyrics, rap, epic, cinematic</t>
+        </is>
+      </c>
+      <c r="J3" s="15" t="n"/>
+      <c r="K3" s="15" t="n"/>
+      <c r="L3" s="3">
+        <f>TEXT(INT((SUM($J$2:J2)*60+SUM($K$2:K2))/60),"0")&amp;":"&amp;TEXT(MOD((SUM($J$2:J2)*60+SUM($K$2:K2)),60),"00")</f>
+        <v/>
+      </c>
+      <c r="M3" s="3">
+        <f>L3&amp;" "&amp;E3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>昼｜森の中を疾走</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>歌</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>105</v>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>急がば回れ、忍者は回って急ぐ</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>ことわざ「急がば回れ」を逆手にとった洒落</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Japanese groove pop, upbeat, bright and refreshing, 105 BPM, punchy drums, funky bassline, Japanese shakuhachi, Japanese shinobue flute, driving rhythm, rushing forest wind, energetic male vocal, Japanese lyrics, Japanese call-and-response chants, male group chorus, head nod</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>[Intro]
+（そーれ　そーれ）
+[Verse]
+すぎの　もりを　かけぬけて
+こけの　いわを　ぽんと　こえ
+えだから　えだへ　とびうつり
+こもれびの　なかを　はしってく
+[Pre-Chorus]
+いそがば　まわれと　いうけれど
+まわって　いそげば　まにあうさ
+[Chorus]
+はしれ（はっ）　はしれ（それ）　もりの　なか
+くるり　まわって　いそいで　いこう
+かぜに　なって（よいしょ）　とりと　ならんで（それ）
+やまの　むこうへ　ひとっとび
+[Instrumental Break]
+[Verse]
+たきの　しぶきを　くぐりぬけ
+しかの　おやこに　あいさつ
+どんぐり　ひろって　ふところへ
+ひるには　さとへ　つくだろう
+[Pre-Chorus]
+いそがば　まわれと　いうけれど
+まわって　いそげば　まにあうさ
+[Chorus]
+はしれ（はっ）　はしれ（それ）　もりの　なか
+くるり　まわって　いそいで　いこう
+かぜに　なって（よいしょ）　とりと　ならんで（それ）
+やまの　むこうへ　ひとっとび
+[Bridge]
+ざわ　ざわ　はっぱが　てを　たたく
+（そーれ）　もっと　はやく
+[Chorus]
+はしれ（はっ）　はしれ（それ）　もりの　なか
+くるり　まわって　いそいで　いこう
+かぜに　なって（よいしょ）　とりと　ならんで（それ）
+やまの　むこうへ　ひとっとび
+[Outro]
+（そーれ）</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
+        <is>
+          <t>dark, horror, scary, English lyrics, rap, epic, cinematic</t>
+        </is>
+      </c>
+      <c r="J4" s="15" t="n"/>
+      <c r="K4" s="15" t="n"/>
+      <c r="L4" s="3">
+        <f>TEXT(INT((SUM($J$2:J3)*60+SUM($K$2:K3))/60),"0")&amp;":"&amp;TEXT(MOD((SUM($J$2:J3)*60+SUM($K$2:K3)),60),"00")</f>
+        <v/>
+      </c>
+      <c r="M4" s="3">
+        <f>L4&amp;" "&amp;E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>ひと休み｜竹林で尺八の独奏</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>インスト</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>96</v>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>竹を割ったような、まっすぐな尺八</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>慣用句「竹を割ったような（さっぱりした）」×竹でできた尺八</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>Japanese groove instrumental, upbeat, bright and refreshing, 96 BPM, punchy drums, funky bassline, long expressive Japanese shakuhachi solo as the lead melody, Japanese koto accompaniment, light Japanese shamisen, head nod, extended arrangement, no vocals, instrumental</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>（Instrumental をオンにする。歌詞欄は使わない）</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>vocals, singing, dark, horror, scary, epic, cinematic</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="n"/>
+      <c r="K5" s="15" t="n"/>
+      <c r="L5" s="3">
+        <f>TEXT(INT((SUM($J$2:J4)*60+SUM($K$2:K4))/60),"0")&amp;":"&amp;TEXT(MOD((SUM($J$2:J4)*60+SUM($K$2:K4)),60),"00")</f>
+        <v/>
+      </c>
+      <c r="M5" s="3">
+        <f>L5&amp;" "&amp;E5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>夕方｜屋根の上で町を見下ろす</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>歌</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>猫の額ほどの屋根で、天下をとる</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>慣用句「猫の額（とても狭い）」×天下とり</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>Japanese groove pop, upbeat, bright and refreshing, 98 BPM, punchy drums, funky bassline, Japanese shakuhachi, Japanese shamisen, warm sunset groove, energetic male vocal, Japanese lyrics, Japanese call-and-response chants, male group chorus, head nod</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>[Intro]
+（いよっ）
+[Verse]
+ゆうやけ　いろの　かわらやね
+ねこと　ならんで　すわったら
+とおくの　しろも　ちいさくて
+てのひらに　のりそうだ
+[Pre-Chorus]
+ねこの　ひたいほどの　ばしょだけど
+ここが　おいらの　とくとうせき
+[Chorus]
+いよっ（はっ）　てんか（それ）　とったぞ
+やねの　うえから　まちを　みおろす
+てを　ふって（よいしょ）　くびを　ふって（それ）
+ゆうひと　いっしょに　おどろうよ
+[Instrumental Break]
+[Verse]
+えんとつ　けむりが　ゆらゆらと
+ごはんの　においが　のぼってくる
+ちょうちん　ぽつぽつ　ともりだし
+まちが　よるへと　きがえてく
+[Pre-Chorus]
+ねこの　ひたいほどの　ばしょだけど
+ここが　おいらの　とくとうせき
+[Chorus]
+いよっ（はっ）　てんか（それ）　とったぞ
+やねの　うえから　まちを　みおろす
+てを　ふって（よいしょ）　くびを　ふって（それ）
+ゆうひと　いっしょに　おどろうよ
+[Bridge]
+（にゃあ）と　ねこが　あいのて　いれて
+ふたりで　そろって　もういっかい
+[Chorus]
+いよっ（はっ）　てんか（それ）　とったぞ
+やねの　うえから　まちを　みおろす
+てを　ふって（よいしょ）　くびを　ふって（それ）
+ゆうひと　いっしょに　おどろうよ
+[Outro]
+（にゃあ）</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>dark, horror, scary, English lyrics, rap, epic, cinematic</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="n"/>
+      <c r="K6" s="15" t="n"/>
+      <c r="L6" s="3">
+        <f>TEXT(INT((SUM($J$2:J5)*60+SUM($K$2:K5))/60),"0")&amp;":"&amp;TEXT(MOD((SUM($J$2:J5)*60+SUM($K$2:K5)),60),"00")</f>
+        <v/>
+      </c>
+      <c r="M6" s="3">
+        <f>L6&amp;" "&amp;E6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>夜｜満月の屋根でお月見（少し落ち着く曲）</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>歌</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>花より団子、満月より月見団子</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>ことわざ「花より団子」×お月見の団子</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>Japanese groove pop, upbeat, bright and refreshing, 90 BPM, punchy drums, funky bassline, Japanese shakuhachi, a little slower and relaxed, warm and cozy, Japanese koto, gentle shakuhachi, energetic male vocal, Japanese lyrics, Japanese call-and-response chants, male group chorus, head nod</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>[Intro]
+（よいしょ）
+[Verse]
+まんまるの　つきが　のぼったら
+すすきが　さらさら　ゆれている
+おだんご　みっつ　ならべたら
+きょうは　しゅぎょうも　おやすみだ
+[Pre-Chorus]
+はなより　だんご　つきより　だんご
+みんなで　わけて　ほおばろう
+[Chorus]
+ぽん　ぽん（はっ）　つきが（それ）　わらってる
+やねの　うえで　ゆっくり　ゆれて
+ひとつ　ふたつ（よいしょ）　おだんご　たべて（それ）
+こよいは　ゆるりと　くびを　ふろう
+[Instrumental Break]
+[Verse]
+むしの　こえが　りん　りん　と
+よかぜに　のって　とどいたら
+ししょうも　めを　ほそめて
+むかしの　はなしを　はじめた
+[Pre-Chorus]
+はなより　だんご　つきより　だんご
+みんなで　わけて　ほおばろう
+[Chorus]
+ぽん　ぽん（はっ）　つきが（それ）　わらってる
+やねの　うえで　ゆっくり　ゆれて
+ひとつ　ふたつ（よいしょ）　おだんご　たべて（それ）
+こよいは　ゆるりと　くびを　ふろう
+[Bridge]
+つきの　うさぎも　もちを　つく
+（ぺったん）（ぺったん）　ゆっくりと
+[Chorus]
+ぽん　ぽん（はっ）　つきが（それ）　わらってる
+やねの　うえで　ゆっくり　ゆれて
+ひとつ　ふたつ（よいしょ）　おだんご　たべて（それ）
+こよいは　ゆるりと　くびを　ふろう
+[Outro]
+（よいしょ）</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>dark, horror, scary, English lyrics, rap, epic, cinematic</t>
+        </is>
+      </c>
+      <c r="J7" s="15" t="n"/>
+      <c r="K7" s="15" t="n"/>
+      <c r="L7" s="3">
+        <f>TEXT(INT((SUM($J$2:J6)*60+SUM($K$2:K6))/60),"0")&amp;":"&amp;TEXT(MOD((SUM($J$2:J6)*60+SUM($K$2:K6)),60),"00")</f>
+        <v/>
+      </c>
+      <c r="M7" s="3">
+        <f>L7&amp;" "&amp;E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>夜明け前｜太鼓と三味線で盛り上げ直す</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>インスト</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>善は急げ、太鼓はもっと急げ</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>ことわざ「善は急げ」のもじり。フィナーレへ向けて加速</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Japanese groove instrumental, upbeat, bright and refreshing, 100 BPM, punchy drums, funky bassline, Japanese taiko drums ensemble breaks, fast Japanese shamisen solo, Japanese shinobue flute, building energy, head nod, extended arrangement, no vocals, instrumental</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>（Instrumental をオンにする。歌詞欄は使わない）</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>vocals, singing, dark, horror, scary, epic, cinematic</t>
+        </is>
+      </c>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="3">
+        <f>TEXT(INT((SUM($J$2:J7)*60+SUM($K$2:K7))/60),"0")&amp;":"&amp;TEXT(MOD((SUM($J$2:J7)*60+SUM($K$2:K7)),60),"00")</f>
+        <v/>
+      </c>
+      <c r="M8" s="3">
+        <f>L8&amp;" "&amp;E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>フィナーレ｜ふたたび朝の屋根へ</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>歌</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>終わりよければ、夜明けもよし</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>ことわざ「終わりよければ全てよし」。1曲目のサビが戻ってくる</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>Japanese groove pop, upbeat, bright and refreshing, 102 BPM, punchy drums, funky bassline, Japanese shakuhachi, Japanese shamisen, taiko drums, big joyful finale feeling, sunrise, energetic male vocal, Japanese lyrics, Japanese call-and-response chants, male group chorus, head nod</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>[Intro]
+（そーれ）
+[Verse]
+よるの　とばりが　うすれていく
+しゅりけん　もりみち　まんげつも
+ぜんぶ　ふところに　しまいこみ
+また　あの　やねへと　かえってきた
+[Pre-Chorus]
+おわり　よければ　すべて　よし
+さあ　みんなで　うたおうよ
+[Chorus]
+はやおき（はっ）　さんもん（それ）　とくを　する
+やねの　うえなら　ごもんの　とく
+あさひに（よいしょ）　てを　のばせ（それ）
+あしたも　ここで　あおうじゃないか
+[Instrumental Break]
+[Verse]
+みならいも　ししょうも　ねこも
+ならんで　あさひを　あびている
+ほら　まちが　めを　さましたら
+きょうも　いちにち　はじまるよ
+[Pre-Chorus]
+おわり　よければ　すべて　よし
+さあ　みんなで　うたおうよ
+[Chorus]
+はやおき（はっ）　さんもん（それ）　とくを　する
+やねの　うえなら　ごもんの　とく
+あさひに（よいしょ）　てを　のばせ（それ）
+あしたも　ここで　あおうじゃないか
+[Bridge]
+いよっ（いよっ）　そーれ（そーれ）
+いよっ（いよっ）　そーれ（そーれ）
+[Chorus]
+はやおき（はっ）　さんもん（それ）　とくを　する
+やねの　うえなら　ごもんの　とく
+あさひに（よいしょ）　てを　のばせ（それ）
+あしたも　ここで　あおうじゃないか
+[Outro]
+（そーれ）</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>dark, horror, scary, English lyrics, rap, epic, cinematic</t>
+        </is>
+      </c>
+      <c r="J9" s="15" t="n"/>
+      <c r="K9" s="15" t="n"/>
+      <c r="L9" s="3">
+        <f>TEXT(INT((SUM($J$2:J8)*60+SUM($K$2:K8))/60),"0")&amp;":"&amp;TEXT(MOD((SUM($J$2:J8)*60+SUM($K$2:K8)),60),"00")</f>
+        <v/>
+      </c>
+      <c r="M9" s="3">
+        <f>L9&amp;" "&amp;E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr"/>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>合計の長さ</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11">
+        <f>TEXT(INT((SUM(J2:J9)*60+SUM(K2:K9))/60),"0")&amp;":"&amp;TEXT(MOD((SUM(J2:J9)*60+SUM(K2:K9)),60),"00")</f>
+        <v/>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>（30分前後が目安）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="n"/>
+      <c r="B12" s="17" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>動画タイトル（コピペ）</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>忍ぶれど、ビートに出にけり屋根の上｜和風 Jazzy HipHop｜作業・通勤・ドライブBGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>使い方</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>1. 曲ごとに①②③④をSunoに貼って生成（インスト曲は Instrumental をオン）。3分未満なら Extend で伸ばす</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr"/>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>2. できた曲の長さを黄色のセル（分・秒）に入れると、タイムスタンプと⑤の概要欄リストが自動で出る</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr"/>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>3. ⑤の列を上から下までコピーして、YouTubeの概要欄に貼る（0:00から始まるので章分けもされる）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>雰囲気をそろえるコツ</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Style欄の前半（Japanese groove pop〜shakuhachi）は全曲共通。曲ごとに変えているのは後半の楽器と場面だけ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>リピートする場合</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>2周目は曲順を少し入れ替えると安心（例：1→3→2→5→4→6→7→8）。そのときはタイムスタンプも周回分を足す</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B15:I15"/>
+    <mergeCell ref="B11:I11"/>
+    <mergeCell ref="B16:I16"/>
+    <mergeCell ref="B14:I14"/>
+    <mergeCell ref="B17:I17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00548235"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1600,7 +2481,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4016,7 +4897,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4444,7 +5325,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5023,7 +5904,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>